<commit_message>
Update LISTS_OF_CITATIONS, images, and citations.xlsx
</commit_message>
<xml_diff>
--- a/community/citations.xlsx
+++ b/community/citations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PD5W\Downloads\BOT\3W\community\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67B198D1-B4F6-4099-9633-3F7C876A9178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02626C3D-FE97-4D3C-AA8D-0C8A8ADEC9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C98DDA46-7193-4817-99A0-E7574FD64AD0}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3953" uniqueCount="1216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3953" uniqueCount="1215">
   <si>
     <t>ID</t>
   </si>
@@ -3353,9 +3353,6 @@
   </si>
   <si>
     <t>Machine Learning-Based Intelligent Measurement in Industrial Digital Twins</t>
-  </si>
-  <si>
-    <t>Conference Paper</t>
   </si>
   <si>
     <t>http://doi.org/10.1007/978-3-032-13612-1_2</t>
@@ -5019,13 +5016,13 @@
         <v>18</v>
       </c>
       <c r="B19" s="20" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C19" s="18" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="D19" s="20" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="E19" s="20" t="s">
         <v>20</v>
@@ -5034,10 +5031,10 @@
         <v>2020</v>
       </c>
       <c r="G19" s="20" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="H19" s="35" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
@@ -5045,25 +5042,25 @@
         <v>19</v>
       </c>
       <c r="B20" s="20" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="C20" s="18" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="D20" s="20" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F20" s="34">
         <v>2020</v>
       </c>
       <c r="G20" s="20" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="H20" s="35" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
@@ -6111,25 +6108,25 @@
         <v>60</v>
       </c>
       <c r="B61" s="20" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="C61" s="18" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="D61" s="20" t="s">
         <v>39</v>
       </c>
       <c r="E61" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F61" s="34">
         <v>2022</v>
       </c>
       <c r="G61" s="20" t="s">
+        <v>1148</v>
+      </c>
+      <c r="H61" s="35" t="s">
         <v>1149</v>
-      </c>
-      <c r="H61" s="35" t="s">
-        <v>1150</v>
       </c>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
@@ -6137,25 +6134,25 @@
         <v>61</v>
       </c>
       <c r="B62" s="20" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="C62" s="18" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="D62" s="20" t="s">
         <v>39</v>
       </c>
       <c r="E62" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F62" s="34">
         <v>2022</v>
       </c>
       <c r="G62" s="20" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="H62" s="35" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
@@ -6163,13 +6160,13 @@
         <v>62</v>
       </c>
       <c r="B63" s="20" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="C63" s="18" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="D63" s="20" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="E63" s="20" t="s">
         <v>20</v>
@@ -6178,10 +6175,10 @@
         <v>2022</v>
       </c>
       <c r="G63" s="20" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="H63" s="35" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
@@ -6839,25 +6836,25 @@
         <v>88</v>
       </c>
       <c r="B89" s="20" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="C89" s="18" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="D89" s="20" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="E89" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F89" s="34">
         <v>2023</v>
       </c>
       <c r="G89" s="20" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="H89" s="35" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -7333,25 +7330,25 @@
         <v>107</v>
       </c>
       <c r="B108" s="20" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="C108" s="18" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="D108" s="20" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="E108" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F108" s="34">
         <v>2024</v>
       </c>
       <c r="G108" s="20" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="H108" s="35" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="109" spans="1:8" s="31" customFormat="1" x14ac:dyDescent="0.25">
@@ -7359,13 +7356,13 @@
         <v>108</v>
       </c>
       <c r="B109" s="20" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="C109" s="18" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="D109" s="20" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="E109" s="20" t="s">
         <v>20</v>
@@ -7374,10 +7371,10 @@
         <v>2024</v>
       </c>
       <c r="G109" s="20" t="s">
+        <v>1133</v>
+      </c>
+      <c r="H109" s="35" t="s">
         <v>1134</v>
-      </c>
-      <c r="H109" s="35" t="s">
-        <v>1135</v>
       </c>
     </row>
     <row r="110" spans="1:8" s="31" customFormat="1" x14ac:dyDescent="0.25">
@@ -7385,25 +7382,25 @@
         <v>109</v>
       </c>
       <c r="B110" s="20" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="C110" s="18" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="D110" s="20" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="E110" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F110" s="34">
         <v>2024</v>
       </c>
       <c r="G110" s="20" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="H110" s="35" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="111" spans="1:8" s="31" customFormat="1" x14ac:dyDescent="0.25">
@@ -7871,7 +7868,7 @@
         <v>926</v>
       </c>
       <c r="H128" s="35" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.25">
@@ -7923,7 +7920,7 @@
         <v>989</v>
       </c>
       <c r="H130" s="35" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
@@ -7975,7 +7972,7 @@
         <v>1011</v>
       </c>
       <c r="H132" s="35" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
     </row>
     <row r="133" spans="1:8" x14ac:dyDescent="0.25">
@@ -7983,13 +7980,13 @@
         <v>132</v>
       </c>
       <c r="B133" s="20" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="C133" s="18" t="s">
+        <v>1072</v>
+      </c>
+      <c r="D133" s="20" t="s">
         <v>1073</v>
-      </c>
-      <c r="D133" s="20" t="s">
-        <v>1074</v>
       </c>
       <c r="E133" s="20" t="s">
         <v>20</v>
@@ -7998,10 +7995,10 @@
         <v>2025</v>
       </c>
       <c r="G133" s="20" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="H133" s="35" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.25">
@@ -8009,25 +8006,25 @@
         <v>133</v>
       </c>
       <c r="B134" s="20" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="C134" s="18" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="D134" s="20" t="s">
         <v>85</v>
       </c>
       <c r="E134" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F134" s="34">
         <v>2025</v>
       </c>
       <c r="G134" s="20" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="H134" s="35" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.25">
@@ -8035,13 +8032,13 @@
         <v>134</v>
       </c>
       <c r="B135" s="20" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="C135" s="18" t="s">
+        <v>1089</v>
+      </c>
+      <c r="D135" s="20" t="s">
         <v>1090</v>
-      </c>
-      <c r="D135" s="20" t="s">
-        <v>1091</v>
       </c>
       <c r="E135" s="20" t="s">
         <v>20</v>
@@ -8050,10 +8047,10 @@
         <v>2025</v>
       </c>
       <c r="G135" s="20" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="H135" s="35" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
     </row>
     <row r="136" spans="1:8" x14ac:dyDescent="0.25">
@@ -8061,13 +8058,13 @@
         <v>135</v>
       </c>
       <c r="B136" s="20" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C136" s="18" t="s">
+        <v>1107</v>
+      </c>
+      <c r="D136" s="20" t="s">
         <v>1128</v>
-      </c>
-      <c r="C136" s="18" t="s">
-        <v>1108</v>
-      </c>
-      <c r="D136" s="20" t="s">
-        <v>1129</v>
       </c>
       <c r="E136" s="20" t="s">
         <v>20</v>
@@ -8076,10 +8073,10 @@
         <v>2025</v>
       </c>
       <c r="G136" s="20" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="H136" s="35" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="137" spans="1:8" x14ac:dyDescent="0.25">
@@ -8087,25 +8084,25 @@
         <v>136</v>
       </c>
       <c r="B137" s="20" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="C137" s="18" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="D137" s="20" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="E137" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F137" s="34">
         <v>2025</v>
       </c>
       <c r="G137" s="20" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="H137" s="35" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
     </row>
     <row r="138" spans="1:8" x14ac:dyDescent="0.25">
@@ -8113,25 +8110,25 @@
         <v>137</v>
       </c>
       <c r="B138" s="20" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C138" s="18" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="D138" s="20" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="E138" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F138" s="34">
         <v>2025</v>
       </c>
       <c r="G138" s="20" t="s">
+        <v>1182</v>
+      </c>
+      <c r="H138" s="35" t="s">
         <v>1183</v>
-      </c>
-      <c r="H138" s="35" t="s">
-        <v>1184</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.25">
@@ -8139,25 +8136,25 @@
         <v>138</v>
       </c>
       <c r="B139" s="20" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C139" s="18" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="D139" s="20" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="E139" s="20" t="s">
-        <v>1062</v>
+        <v>10</v>
       </c>
       <c r="F139" s="34">
         <v>2025</v>
       </c>
       <c r="G139" s="20" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="H139" s="35" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
     </row>
     <row r="140" spans="1:8" x14ac:dyDescent="0.25">
@@ -8313,7 +8310,7 @@
         <v>1009</v>
       </c>
       <c r="H145" s="35" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.25">
@@ -8347,7 +8344,7 @@
         <v>146</v>
       </c>
       <c r="B147" s="20" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="C147" s="18" t="s">
         <v>1061</v>
@@ -8362,16 +8359,14 @@
         <v>2026</v>
       </c>
       <c r="G147" s="20" t="s">
+        <v>1062</v>
+      </c>
+      <c r="H147" s="35" t="s">
         <v>1063</v>
       </c>
-      <c r="H147" s="35" t="s">
-        <v>1064</v>
-      </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A148" s="33">
-        <v>147</v>
-      </c>
+      <c r="A148" s="33"/>
       <c r="B148" s="20"/>
       <c r="D148" s="20"/>
       <c r="E148" s="20"/>
@@ -8380,9 +8375,7 @@
       <c r="H148" s="35"/>
     </row>
     <row r="149" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A149" s="33">
-        <v>148</v>
-      </c>
+      <c r="A149" s="33"/>
       <c r="B149" s="20"/>
       <c r="D149" s="20"/>
       <c r="E149" s="20"/>
@@ -8391,9 +8384,7 @@
       <c r="H149" s="35"/>
     </row>
     <row r="150" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A150" s="33">
-        <v>149</v>
-      </c>
+      <c r="A150" s="33"/>
       <c r="B150" s="20"/>
       <c r="D150" s="20"/>
       <c r="E150" s="20"/>
@@ -8402,9 +8393,7 @@
       <c r="H150" s="35"/>
     </row>
     <row r="151" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A151" s="33">
-        <v>150</v>
-      </c>
+      <c r="A151" s="33"/>
       <c r="B151" s="20"/>
       <c r="D151" s="20"/>
       <c r="E151" s="20"/>
@@ -8413,9 +8402,7 @@
       <c r="H151" s="35"/>
     </row>
     <row r="152" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A152" s="33">
-        <v>151</v>
-      </c>
+      <c r="A152" s="33"/>
       <c r="B152" s="20"/>
       <c r="D152" s="20"/>
       <c r="E152" s="20"/>
@@ -8424,9 +8411,7 @@
       <c r="H152" s="35"/>
     </row>
     <row r="153" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A153" s="33">
-        <v>152</v>
-      </c>
+      <c r="A153" s="33"/>
       <c r="B153" s="20"/>
       <c r="D153" s="20"/>
       <c r="E153" s="20"/>
@@ -8435,9 +8420,7 @@
       <c r="H153" s="35"/>
     </row>
     <row r="154" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A154" s="33">
-        <v>153</v>
-      </c>
+      <c r="A154" s="33"/>
       <c r="B154" s="20"/>
       <c r="D154" s="20"/>
       <c r="E154" s="20"/>
@@ -8446,9 +8429,7 @@
       <c r="H154" s="35"/>
     </row>
     <row r="155" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A155" s="33">
-        <v>154</v>
-      </c>
+      <c r="A155" s="33"/>
       <c r="B155" s="20"/>
       <c r="D155" s="20"/>
       <c r="E155" s="20"/>
@@ -8457,9 +8438,7 @@
       <c r="H155" s="35"/>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A156" s="33">
-        <v>155</v>
-      </c>
+      <c r="A156" s="33"/>
       <c r="B156" s="20"/>
       <c r="D156" s="20"/>
       <c r="E156" s="20"/>
@@ -8468,9 +8447,7 @@
       <c r="H156" s="35"/>
     </row>
     <row r="157" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A157" s="33">
-        <v>156</v>
-      </c>
+      <c r="A157" s="33"/>
       <c r="B157" s="20"/>
       <c r="D157" s="20"/>
       <c r="E157" s="20"/>
@@ -8479,9 +8456,7 @@
       <c r="H157" s="35"/>
     </row>
     <row r="158" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A158" s="33">
-        <v>157</v>
-      </c>
+      <c r="A158" s="33"/>
       <c r="B158" s="20"/>
       <c r="D158" s="20"/>
       <c r="E158" s="20"/>
@@ -8490,9 +8465,7 @@
       <c r="H158" s="35"/>
     </row>
     <row r="159" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A159" s="33">
-        <v>158</v>
-      </c>
+      <c r="A159" s="33"/>
       <c r="B159" s="20"/>
       <c r="D159" s="20"/>
       <c r="E159" s="20"/>
@@ -8501,9 +8474,7 @@
       <c r="H159" s="35"/>
     </row>
     <row r="160" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A160" s="33">
-        <v>159</v>
-      </c>
+      <c r="A160" s="33"/>
       <c r="B160" s="20"/>
       <c r="D160" s="20"/>
       <c r="E160" s="20"/>
@@ -8512,9 +8483,7 @@
       <c r="H160" s="35"/>
     </row>
     <row r="161" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A161" s="33">
-        <v>160</v>
-      </c>
+      <c r="A161" s="33"/>
       <c r="B161" s="20"/>
       <c r="D161" s="20"/>
       <c r="E161" s="20"/>
@@ -8523,9 +8492,7 @@
       <c r="H161" s="35"/>
     </row>
     <row r="162" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A162" s="36">
-        <v>161</v>
-      </c>
+      <c r="A162" s="36"/>
       <c r="B162" s="37"/>
       <c r="C162" s="38"/>
       <c r="D162" s="37"/>
@@ -8576,7 +8543,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="43" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>411</v>
@@ -8586,7 +8553,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="44" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -8666,17 +8633,17 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C8" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A8)</f>
         <v>1</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -8756,7 +8723,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>1046</v>
@@ -8766,7 +8733,7 @@
         <v>1</v>
       </c>
       <c r="D14" s="14" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -8891,7 +8858,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>526</v>
@@ -8901,12 +8868,12 @@
         <v>1</v>
       </c>
       <c r="D23" s="14" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>422</v>
@@ -8966,17 +8933,17 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C28" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A28)</f>
         <v>1</v>
       </c>
       <c r="D28" s="14" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
@@ -9021,7 +8988,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -9071,7 +9038,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>422</v>
@@ -9086,7 +9053,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>526</v>
@@ -9096,12 +9063,12 @@
         <v>1</v>
       </c>
       <c r="D36" s="14" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>526</v>
@@ -9111,7 +9078,7 @@
         <v>1</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
@@ -9131,7 +9098,7 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="B39" s="4" t="s">
         <v>422</v>
@@ -9281,7 +9248,7 @@
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>422</v>
@@ -9311,17 +9278,17 @@
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
+        <v>1077</v>
+      </c>
+      <c r="B51" s="4" t="s">
         <v>1078</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>1079</v>
       </c>
       <c r="C51" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A51)</f>
         <v>1</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
@@ -9386,7 +9353,7 @@
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>422</v>
@@ -9731,7 +9698,7 @@
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>422</v>
@@ -9741,7 +9708,7 @@
         <v>1</v>
       </c>
       <c r="D79" s="14" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
@@ -9851,7 +9818,7 @@
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" s="3" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>422</v>
@@ -9861,7 +9828,7 @@
         <v>1</v>
       </c>
       <c r="D87" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
@@ -9986,7 +9953,7 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="B96" s="4" t="s">
         <v>469</v>
@@ -9996,22 +9963,22 @@
         <v>1</v>
       </c>
       <c r="D96" s="14" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C97" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A97)</f>
         <v>1</v>
       </c>
       <c r="D97" s="14" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
@@ -10031,7 +9998,7 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B99" s="4" t="s">
         <v>422</v>
@@ -10061,7 +10028,7 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B101" s="4" t="s">
         <v>526</v>
@@ -10071,7 +10038,7 @@
         <v>1</v>
       </c>
       <c r="D101" s="14" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
@@ -10106,7 +10073,7 @@
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="B104" s="4" t="s">
         <v>422</v>
@@ -10116,7 +10083,7 @@
         <v>1</v>
       </c>
       <c r="D104" s="14" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -10206,7 +10173,7 @@
         <v>5</v>
       </c>
       <c r="D110" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.25">
@@ -10236,7 +10203,7 @@
         <v>1</v>
       </c>
       <c r="D112" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.25">
@@ -10301,7 +10268,7 @@
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="B117" s="4" t="s">
         <v>422</v>
@@ -10316,7 +10283,7 @@
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B118" s="4" t="s">
         <v>422</v>
@@ -10586,7 +10553,7 @@
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="B136" s="4" t="s">
         <v>422</v>
@@ -10601,7 +10568,7 @@
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B137" s="4" t="s">
         <v>526</v>
@@ -10611,7 +10578,7 @@
         <v>1</v>
       </c>
       <c r="D137" s="14" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.25">
@@ -10676,7 +10643,7 @@
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A142" s="3" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B142" s="4" t="s">
         <v>422</v>
@@ -10686,12 +10653,12 @@
         <v>1</v>
       </c>
       <c r="D142" s="14" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A143" s="3" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="B143" s="4" t="s">
         <v>526</v>
@@ -10701,7 +10668,7 @@
         <v>1</v>
       </c>
       <c r="D143" s="14" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.25">
@@ -10751,7 +10718,7 @@
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A147" s="3" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="B147" s="4" t="s">
         <v>422</v>
@@ -10791,7 +10758,7 @@
         <v>1</v>
       </c>
       <c r="D149" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.25">
@@ -10961,7 +10928,7 @@
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A161" s="3" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="B161" s="4" t="s">
         <v>422</v>
@@ -10976,7 +10943,7 @@
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A162" s="3" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="B162" s="4" t="s">
         <v>526</v>
@@ -10986,7 +10953,7 @@
         <v>1</v>
       </c>
       <c r="D162" s="14" t="s">
-        <v>1069</v>
+        <v>1068</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.25">
@@ -11151,7 +11118,7 @@
         <v>4</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="174" spans="1:4" x14ac:dyDescent="0.25">
@@ -11306,7 +11273,7 @@
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A184" s="3" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B184" s="4" t="s">
         <v>422</v>
@@ -11316,7 +11283,7 @@
         <v>1</v>
       </c>
       <c r="D184" s="14" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="185" spans="1:4" x14ac:dyDescent="0.25">
@@ -11426,7 +11393,7 @@
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A192" s="3" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B192" s="4" t="s">
         <v>422</v>
@@ -11436,7 +11403,7 @@
         <v>1</v>
       </c>
       <c r="D192" s="14" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.25">
@@ -11576,7 +11543,7 @@
     </row>
     <row r="202" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A202" s="3" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B202" s="4" t="s">
         <v>422</v>
@@ -11661,7 +11628,7 @@
         <v>1</v>
       </c>
       <c r="D207" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.25">
@@ -11741,7 +11708,7 @@
     </row>
     <row r="213" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A213" s="3" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B213" s="4" t="s">
         <v>422</v>
@@ -11786,7 +11753,7 @@
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A216" s="3" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="B216" s="4" t="s">
         <v>422</v>
@@ -11796,12 +11763,12 @@
         <v>1</v>
       </c>
       <c r="D216" s="14" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A217" s="3" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="B217" s="4" t="s">
         <v>422</v>
@@ -11811,12 +11778,12 @@
         <v>1</v>
       </c>
       <c r="D217" s="14" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A218" s="3" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="B218" s="4" t="s">
         <v>422</v>
@@ -11826,7 +11793,7 @@
         <v>1</v>
       </c>
       <c r="D218" s="14" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.25">
@@ -11856,7 +11823,7 @@
         <v>1</v>
       </c>
       <c r="D220" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.25">
@@ -11876,7 +11843,7 @@
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A222" s="3" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="B222" s="4" t="s">
         <v>422</v>
@@ -11886,7 +11853,7 @@
         <v>1</v>
       </c>
       <c r="D222" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="223" spans="1:4" x14ac:dyDescent="0.25">
@@ -12071,7 +12038,7 @@
     </row>
     <row r="235" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A235" s="3" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="B235" s="4" t="s">
         <v>526</v>
@@ -12081,12 +12048,12 @@
         <v>1</v>
       </c>
       <c r="D235" s="14" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="236" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A236" s="3" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="B236" s="4" t="s">
         <v>422</v>
@@ -12096,7 +12063,7 @@
         <v>1</v>
       </c>
       <c r="D236" s="14" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
     </row>
     <row r="237" spans="1:4" x14ac:dyDescent="0.25">
@@ -12236,17 +12203,17 @@
     </row>
     <row r="246" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A246" s="3" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="B246" s="4" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C246" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A246)</f>
         <v>1</v>
       </c>
       <c r="D246" s="14" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="247" spans="1:4" x14ac:dyDescent="0.25">
@@ -12296,7 +12263,7 @@
     </row>
     <row r="250" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A250" s="3" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="B250" s="4" t="s">
         <v>422</v>
@@ -12306,7 +12273,7 @@
         <v>1</v>
       </c>
       <c r="D250" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="251" spans="1:4" x14ac:dyDescent="0.25">
@@ -12336,7 +12303,7 @@
         <v>2</v>
       </c>
       <c r="D252" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="253" spans="1:4" x14ac:dyDescent="0.25">
@@ -12356,17 +12323,17 @@
     </row>
     <row r="254" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A254" s="3" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="B254" s="4" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C254" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A254)</f>
         <v>1</v>
       </c>
       <c r="D254" s="14" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="255" spans="1:4" x14ac:dyDescent="0.25">
@@ -12491,7 +12458,7 @@
     </row>
     <row r="263" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A263" s="3" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="B263" s="4" t="s">
         <v>422</v>
@@ -12521,7 +12488,7 @@
     </row>
     <row r="265" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A265" s="3" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="B265" s="4" t="s">
         <v>422</v>
@@ -12551,7 +12518,7 @@
     </row>
     <row r="267" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A267" s="3" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="B267" s="4" t="s">
         <v>422</v>
@@ -12941,7 +12908,7 @@
     </row>
     <row r="293" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A293" s="3" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="B293" s="4" t="s">
         <v>1046</v>
@@ -12951,7 +12918,7 @@
         <v>1</v>
       </c>
       <c r="D293" s="14" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="294" spans="1:4" x14ac:dyDescent="0.25">
@@ -13046,7 +13013,7 @@
     </row>
     <row r="300" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A300" s="3" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="B300" s="4" t="s">
         <v>526</v>
@@ -13056,7 +13023,7 @@
         <v>1</v>
       </c>
       <c r="D300" s="14" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="301" spans="1:4" x14ac:dyDescent="0.25">
@@ -13116,7 +13083,7 @@
         <v>3</v>
       </c>
       <c r="D304" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="305" spans="1:4" x14ac:dyDescent="0.25">
@@ -13236,7 +13203,7 @@
         <v>5</v>
       </c>
       <c r="D312" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="313" spans="1:4" x14ac:dyDescent="0.25">
@@ -13601,7 +13568,7 @@
     </row>
     <row r="337" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A337" s="3" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="B337" s="4" t="s">
         <v>1046</v>
@@ -13611,12 +13578,12 @@
         <v>1</v>
       </c>
       <c r="D337" s="14" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="338" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A338" s="3" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="B338" s="4" t="s">
         <v>411</v>
@@ -13626,12 +13593,12 @@
         <v>1</v>
       </c>
       <c r="D338" s="14" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
     </row>
     <row r="339" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A339" s="3" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="B339" s="4" t="s">
         <v>1046</v>
@@ -13641,7 +13608,7 @@
         <v>1</v>
       </c>
       <c r="D339" s="14" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="340" spans="1:4" x14ac:dyDescent="0.25">
@@ -13661,7 +13628,7 @@
     </row>
     <row r="341" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A341" s="3" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B341" s="4" t="s">
         <v>422</v>
@@ -13721,7 +13688,7 @@
     </row>
     <row r="345" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A345" s="3" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="B345" s="4" t="s">
         <v>469</v>
@@ -13751,7 +13718,7 @@
     </row>
     <row r="347" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A347" s="3" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="B347" s="4" t="s">
         <v>526</v>
@@ -13761,7 +13728,7 @@
         <v>1</v>
       </c>
       <c r="D347" s="14" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
     </row>
     <row r="348" spans="1:4" x14ac:dyDescent="0.25">
@@ -13811,7 +13778,7 @@
     </row>
     <row r="351" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A351" s="3" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="B351" s="4" t="s">
         <v>422</v>
@@ -13841,17 +13808,17 @@
     </row>
     <row r="353" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A353" s="3" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="B353" s="4" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="C353" s="15">
         <f>COUNTIF(citations3!$B$2:$U$208,citations2!A353)</f>
         <v>1</v>
       </c>
       <c r="D353" s="14" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="354" spans="1:4" x14ac:dyDescent="0.25">
@@ -14046,7 +14013,7 @@
         <v>1</v>
       </c>
       <c r="D366" s="14" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="367" spans="1:4" x14ac:dyDescent="0.25">
@@ -14276,7 +14243,7 @@
     </row>
     <row r="382" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A382" s="3" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="B382" s="4" t="s">
         <v>411</v>
@@ -14286,7 +14253,7 @@
         <v>1</v>
       </c>
       <c r="D382" s="14" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
     </row>
     <row r="383" spans="1:4" x14ac:dyDescent="0.25">
@@ -14381,7 +14348,7 @@
     </row>
     <row r="389" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A389" s="3" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="B389" s="4" t="s">
         <v>469</v>
@@ -15435,7 +15402,7 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>768</v>
@@ -17580,19 +17547,19 @@
         <v>60</v>
       </c>
       <c r="B61" s="3" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C61" s="4" t="s">
         <v>1144</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="D61" t="s">
         <v>1145</v>
       </c>
-      <c r="D61" t="s">
+      <c r="E61" s="4" t="s">
         <v>1146</v>
       </c>
-      <c r="E61" s="4" t="s">
+      <c r="F61" t="s">
         <v>1147</v>
-      </c>
-      <c r="F61" t="s">
-        <v>1148</v>
       </c>
       <c r="G61" s="4"/>
       <c r="I61" s="4"/>
@@ -17620,13 +17587,13 @@
         <v>636</v>
       </c>
       <c r="E62" s="4" t="s">
+        <v>1164</v>
+      </c>
+      <c r="F62" t="s">
         <v>1165</v>
       </c>
-      <c r="F62" t="s">
+      <c r="G62" s="4" t="s">
         <v>1166</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>1167</v>
       </c>
       <c r="H62" t="s">
         <v>637</v>
@@ -17635,13 +17602,13 @@
         <v>427</v>
       </c>
       <c r="J62" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="K62" s="4" t="s">
         <v>519</v>
       </c>
       <c r="L62" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="M62" s="4"/>
       <c r="O62" s="4"/>
@@ -17663,7 +17630,7 @@
         <v>525</v>
       </c>
       <c r="D63" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="E63" s="4"/>
       <c r="G63" s="4"/>
@@ -19008,22 +18975,22 @@
         <v>88</v>
       </c>
       <c r="B89" s="3" t="s">
+        <v>1204</v>
+      </c>
+      <c r="C89" s="4" t="s">
         <v>1205</v>
       </c>
-      <c r="C89" s="4" t="s">
+      <c r="D89" t="s">
         <v>1206</v>
       </c>
-      <c r="D89" t="s">
+      <c r="E89" s="4" t="s">
+        <v>1203</v>
+      </c>
+      <c r="F89" t="s">
         <v>1207</v>
       </c>
-      <c r="E89" s="4" t="s">
-        <v>1204</v>
-      </c>
-      <c r="F89" t="s">
+      <c r="G89" s="4" t="s">
         <v>1208</v>
-      </c>
-      <c r="G89" s="4" t="s">
-        <v>1209</v>
       </c>
       <c r="I89" s="4"/>
       <c r="K89" s="4"/>
@@ -19919,22 +19886,22 @@
         <v>108</v>
       </c>
       <c r="B109" s="3" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C109" s="4" t="s">
         <v>1137</v>
       </c>
-      <c r="C109" s="4" t="s">
+      <c r="D109" t="s">
         <v>1138</v>
       </c>
-      <c r="D109" t="s">
+      <c r="E109" s="4" t="s">
         <v>1139</v>
       </c>
-      <c r="E109" s="4" t="s">
+      <c r="F109" t="s">
         <v>1140</v>
       </c>
-      <c r="F109" t="s">
+      <c r="G109" s="4" t="s">
         <v>1141</v>
-      </c>
-      <c r="G109" s="4" t="s">
-        <v>1142</v>
       </c>
       <c r="H109" t="s">
         <v>768</v>
@@ -19972,10 +19939,10 @@
         <v>109</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="D110" t="s">
         <v>480</v>
@@ -21024,13 +20991,13 @@
         <v>132</v>
       </c>
       <c r="B133" s="3" t="s">
+        <v>1075</v>
+      </c>
+      <c r="C133" s="4" t="s">
         <v>1076</v>
       </c>
-      <c r="C133" s="4" t="s">
+      <c r="D133" t="s">
         <v>1077</v>
-      </c>
-      <c r="D133" t="s">
-        <v>1078</v>
       </c>
       <c r="E133" s="4"/>
       <c r="G133" s="4" t="s">
@@ -21072,13 +21039,13 @@
         <v>133</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="C134" s="4" t="s">
         <v>577</v>
       </c>
       <c r="D134" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="E134" s="4" t="s">
         <v>485</v>
@@ -21087,13 +21054,13 @@
         <v>573</v>
       </c>
       <c r="G134" s="4" t="s">
+        <v>1083</v>
+      </c>
+      <c r="H134" t="s">
         <v>1084</v>
       </c>
-      <c r="H134" t="s">
+      <c r="I134" s="4" t="s">
         <v>1085</v>
-      </c>
-      <c r="I134" s="4" t="s">
-        <v>1086</v>
       </c>
       <c r="J134" t="s">
         <v>686</v>
@@ -21105,10 +21072,10 @@
         <v>570</v>
       </c>
       <c r="M134" s="4" t="s">
+        <v>1086</v>
+      </c>
+      <c r="N134" t="s">
         <v>1087</v>
-      </c>
-      <c r="N134" t="s">
-        <v>1088</v>
       </c>
       <c r="O134" s="4" t="s">
         <v>678</v>
@@ -21132,19 +21099,19 @@
         <v>746</v>
       </c>
       <c r="C135" s="4" t="s">
+        <v>1093</v>
+      </c>
+      <c r="D135" t="s">
         <v>1094</v>
       </c>
-      <c r="D135" t="s">
+      <c r="E135" s="4" t="s">
         <v>1095</v>
       </c>
-      <c r="E135" s="4" t="s">
+      <c r="F135" t="s">
         <v>1096</v>
       </c>
-      <c r="F135" t="s">
+      <c r="G135" s="4" t="s">
         <v>1097</v>
-      </c>
-      <c r="G135" s="4" t="s">
-        <v>1098</v>
       </c>
       <c r="H135" t="s">
         <v>737</v>
@@ -21182,16 +21149,16 @@
         <v>135</v>
       </c>
       <c r="B136" s="3" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C136" s="4" t="s">
         <v>1122</v>
       </c>
-      <c r="C136" s="4" t="s">
+      <c r="D136" t="s">
         <v>1123</v>
       </c>
-      <c r="D136" t="s">
+      <c r="E136" s="4" t="s">
         <v>1124</v>
-      </c>
-      <c r="E136" s="4" t="s">
-        <v>1125</v>
       </c>
       <c r="G136" s="4" t="s">
         <v>768</v>
@@ -21232,7 +21199,7 @@
         <v>136</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="C137" s="4" t="s">
         <v>552</v>
@@ -21277,16 +21244,16 @@
         <v>137</v>
       </c>
       <c r="B138" s="3" t="s">
+        <v>1184</v>
+      </c>
+      <c r="C138" s="4" t="s">
         <v>1185</v>
       </c>
-      <c r="C138" s="4" t="s">
+      <c r="D138" t="s">
         <v>1186</v>
       </c>
-      <c r="D138" t="s">
+      <c r="E138" s="4" t="s">
         <v>1187</v>
-      </c>
-      <c r="E138" s="4" t="s">
-        <v>1188</v>
       </c>
       <c r="G138" s="4"/>
       <c r="I138" s="4"/>
@@ -21315,16 +21282,16 @@
         <v>138</v>
       </c>
       <c r="B139" s="3" t="s">
+        <v>1196</v>
+      </c>
+      <c r="C139" s="4" t="s">
         <v>1197</v>
       </c>
-      <c r="C139" s="4" t="s">
+      <c r="D139" t="s">
         <v>1198</v>
       </c>
-      <c r="D139" t="s">
+      <c r="E139" s="4" t="s">
         <v>1199</v>
-      </c>
-      <c r="E139" s="4" t="s">
-        <v>1200</v>
       </c>
       <c r="G139" s="4" t="s">
         <v>768</v>
@@ -21596,13 +21563,13 @@
         <v>146</v>
       </c>
       <c r="B147" s="3" t="s">
+        <v>1065</v>
+      </c>
+      <c r="C147" s="4" t="s">
         <v>1066</v>
       </c>
-      <c r="C147" s="4" t="s">
+      <c r="D147" t="s">
         <v>1067</v>
-      </c>
-      <c r="D147" t="s">
-        <v>1068</v>
       </c>
       <c r="E147" s="4"/>
       <c r="G147" s="4"/>

</xml_diff>